<commit_message>
Replaced unit models with sprites
</commit_message>
<xml_diff>
--- a/Items.xlsx
+++ b/Items.xlsx
@@ -4,7 +4,7 @@
   <fileVersion appName="xl" lastEdited="5" lowestEdited="4" rupBuild="9303"/>
   <workbookPr filterPrivacy="1" defaultThemeVersion="124226"/>
   <bookViews>
-    <workbookView xWindow="240" yWindow="108" windowWidth="14808" windowHeight="8016"/>
+    <workbookView xWindow="240" yWindow="105" windowWidth="14805" windowHeight="8010"/>
   </bookViews>
   <sheets>
     <sheet name="Лист1" sheetId="1" r:id="rId1"/>
@@ -16,7 +16,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="131" uniqueCount="67">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="63">
   <si>
     <t>Name</t>
   </si>
@@ -150,21 +150,9 @@
     <t>Small war hammer</t>
   </si>
   <si>
-    <t>Instantly destroys selected unit</t>
-  </si>
-  <si>
-    <t>Origami</t>
-  </si>
-  <si>
     <t>Additional info</t>
   </si>
   <si>
-    <t>Paper</t>
-  </si>
-  <si>
-    <t>Gains Vulnerable:Fire and Fragile, looses Resistant:Fire, has 1 less maximum health (To a minimum of 1)</t>
-  </si>
-  <si>
     <t>Master bolt</t>
   </si>
   <si>
@@ -174,9 +162,6 @@
     <t>Covers 1 cell in Storm clouds</t>
   </si>
   <si>
-    <t>At the end of the turn, deals 3 (Lightning damage) to units on top</t>
-  </si>
-  <si>
     <t>A critical roll</t>
   </si>
   <si>
@@ -201,9 +186,6 @@
     <t>Randomized</t>
   </si>
   <si>
-    <t>Create a copy of selected unit made out of Paper and place it 2 cells away from the original</t>
-  </si>
-  <si>
     <t>Blood stew</t>
   </si>
   <si>
@@ -217,6 +199,12 @@
   </si>
   <si>
     <t>Applies "Polymorphed" to selected unit</t>
+  </si>
+  <si>
+    <t>Deal 3 (Physical) damage to the target</t>
+  </si>
+  <si>
+    <t>At the end of the round, deals 3 (Lightning damage) to units on top</t>
   </si>
 </sst>
 </file>
@@ -366,7 +354,7 @@
     <xf numFmtId="0" fontId="3" fillId="4" borderId="1" applyNumberFormat="0" applyAlignment="0" applyProtection="0"/>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="0" applyNumberFormat="0" applyBorder="0" applyAlignment="0" applyProtection="0"/>
   </cellStyleXfs>
-  <cellXfs count="24">
+  <cellXfs count="31">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -422,6 +410,15 @@
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="3" fillId="4" borderId="1" xfId="3" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
     <xf numFmtId="0" fontId="4" fillId="5" borderId="2" xfId="4" applyBorder="1" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
@@ -437,6 +434,16 @@
     <xf numFmtId="0" fontId="2" fillId="3" borderId="0" xfId="2" applyAlignment="1">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
     </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="4" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="1" xfId="4" applyBorder="1" applyAlignment="1">
+      <alignment horizontal="center" vertical="center" wrapText="1"/>
+    </xf>
+    <xf numFmtId="0" fontId="4" fillId="5" borderId="0" xfId="4"/>
   </cellXfs>
   <cellStyles count="5">
     <cellStyle name="Вывод" xfId="3" builtinId="21"/>
@@ -743,43 +750,43 @@
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1:M58"/>
-  <sheetFormatPr defaultColWidth="8.88671875" defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultColWidth="8.85546875" defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="1" max="1" width="8.88671875" style="4"/>
+    <col min="1" max="1" width="8.85546875" style="4"/>
     <col min="2" max="2" width="5" style="4" customWidth="1"/>
-    <col min="3" max="3" width="7.88671875" style="4" customWidth="1"/>
-    <col min="4" max="4" width="25.44140625" style="4" customWidth="1"/>
-    <col min="5" max="5" width="3.88671875" style="4" customWidth="1"/>
-    <col min="6" max="6" width="17.33203125" style="4" customWidth="1"/>
-    <col min="7" max="7" width="46.21875" style="4" customWidth="1"/>
-    <col min="8" max="8" width="10.33203125" style="4" customWidth="1"/>
-    <col min="9" max="9" width="40.44140625" style="4" customWidth="1"/>
-    <col min="10" max="10" width="32.44140625" style="4" customWidth="1"/>
-    <col min="11" max="11" width="12.44140625" style="4" customWidth="1"/>
-    <col min="12" max="12" width="8.88671875" style="4"/>
-    <col min="13" max="13" width="5.109375" style="4" customWidth="1"/>
-    <col min="14" max="16384" width="8.88671875" style="4"/>
+    <col min="3" max="3" width="7.85546875" style="4" customWidth="1"/>
+    <col min="4" max="4" width="25.42578125" style="4" customWidth="1"/>
+    <col min="5" max="5" width="3.85546875" style="4" customWidth="1"/>
+    <col min="6" max="6" width="17.28515625" style="4" customWidth="1"/>
+    <col min="7" max="7" width="46.28515625" style="4" customWidth="1"/>
+    <col min="8" max="8" width="10.28515625" style="4" customWidth="1"/>
+    <col min="9" max="9" width="40.42578125" style="4" customWidth="1"/>
+    <col min="10" max="10" width="32.42578125" style="4" customWidth="1"/>
+    <col min="11" max="11" width="12.42578125" style="4" customWidth="1"/>
+    <col min="12" max="12" width="8.85546875" style="4"/>
+    <col min="13" max="13" width="5.140625" style="4" customWidth="1"/>
+    <col min="14" max="16384" width="8.85546875" style="4"/>
   </cols>
   <sheetData>
-    <row r="1" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="A1" s="18" t="s">
+    <row r="1" spans="1:13" ht="14.45" x14ac:dyDescent="0.3">
+      <c r="A1" s="21" t="s">
         <v>5</v>
       </c>
-      <c r="B1" s="18"/>
-      <c r="C1" s="18"/>
-      <c r="D1" s="18"/>
-      <c r="E1" s="18"/>
-      <c r="F1" s="18" t="s">
-        <v>46</v>
-      </c>
-      <c r="G1" s="18"/>
-      <c r="H1" s="18"/>
-      <c r="I1" s="18"/>
-      <c r="J1" s="18"/>
-      <c r="K1" s="18"/>
-      <c r="L1" s="18"/>
-    </row>
-    <row r="4" spans="1:13" x14ac:dyDescent="0.3">
+      <c r="B1" s="21"/>
+      <c r="C1" s="21"/>
+      <c r="D1" s="21"/>
+      <c r="E1" s="21"/>
+      <c r="F1" s="21" t="s">
+        <v>44</v>
+      </c>
+      <c r="G1" s="21"/>
+      <c r="H1" s="21"/>
+      <c r="I1" s="21"/>
+      <c r="J1" s="21"/>
+      <c r="K1" s="21"/>
+      <c r="L1" s="21"/>
+    </row>
+    <row r="4" spans="1:13" ht="14.45" x14ac:dyDescent="0.3">
       <c r="A4" s="1" t="s">
         <v>1</v>
       </c>
@@ -804,7 +811,7 @@
         <v>10</v>
       </c>
     </row>
-    <row r="5" spans="1:13" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="5" spans="1:13" ht="43.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A5" s="2" t="s">
         <v>2</v>
       </c>
@@ -838,7 +845,7 @@
       <c r="I6" s="5"/>
       <c r="J6" s="5"/>
     </row>
-    <row r="7" spans="1:13" ht="16.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="7" spans="1:13" ht="16.149999999999999" customHeight="1" x14ac:dyDescent="0.3">
       <c r="A7" s="3" t="s">
         <v>3</v>
       </c>
@@ -859,7 +866,7 @@
       <c r="I7" s="5"/>
       <c r="J7" s="5"/>
     </row>
-    <row r="8" spans="1:13" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="8" spans="1:13" ht="43.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C8" s="6" t="s">
         <v>6</v>
       </c>
@@ -877,7 +884,7 @@
       <c r="I8" s="5"/>
       <c r="J8" s="5"/>
     </row>
-    <row r="9" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="9" spans="1:13" ht="14.45" x14ac:dyDescent="0.3">
       <c r="C9"/>
       <c r="D9"/>
       <c r="E9" s="5"/>
@@ -887,7 +894,7 @@
       <c r="I9" s="5"/>
       <c r="J9" s="5"/>
     </row>
-    <row r="10" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="10" spans="1:13" ht="14.45" x14ac:dyDescent="0.3">
       <c r="C10" s="6" t="s">
         <v>0</v>
       </c>
@@ -899,7 +906,7 @@
       <c r="I10" s="5"/>
       <c r="J10" s="5"/>
     </row>
-    <row r="11" spans="1:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="11" spans="1:13" ht="28.9" x14ac:dyDescent="0.3">
       <c r="C11" s="6" t="s">
         <v>6</v>
       </c>
@@ -911,13 +918,13 @@
       <c r="I11" s="5"/>
       <c r="J11" s="5"/>
     </row>
-    <row r="12" spans="1:13" x14ac:dyDescent="0.3">
+    <row r="12" spans="1:13" ht="14.45" x14ac:dyDescent="0.3">
       <c r="E12" s="5"/>
       <c r="H12" s="5"/>
       <c r="I12" s="5"/>
       <c r="J12" s="5"/>
     </row>
-    <row r="13" spans="1:13" ht="15" x14ac:dyDescent="0.25">
+    <row r="13" spans="1:13" x14ac:dyDescent="0.25">
       <c r="C13" s="6" t="s">
         <v>0</v>
       </c>
@@ -950,11 +957,11 @@
         <v>26</v>
       </c>
     </row>
-    <row r="14" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C14" s="22" t="s">
+    <row r="14" spans="1:13" ht="30" x14ac:dyDescent="0.25">
+      <c r="C14" s="25" t="s">
         <v>6</v>
       </c>
-      <c r="D14" s="23" t="s">
+      <c r="D14" s="26" t="s">
         <v>19</v>
       </c>
       <c r="E14" s="5"/>
@@ -983,40 +990,40 @@
         <v>15</v>
       </c>
     </row>
-    <row r="15" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C15" s="22"/>
-      <c r="D15" s="23"/>
+    <row r="15" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C15" s="25"/>
+      <c r="D15" s="26"/>
       <c r="E15" s="5"/>
       <c r="F15" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="G15" s="19" t="s">
+      <c r="G15" s="22" t="s">
         <v>31</v>
       </c>
-      <c r="H15" s="20"/>
-      <c r="I15" s="20"/>
-      <c r="J15" s="20"/>
-      <c r="K15" s="20"/>
-      <c r="L15" s="20"/>
-      <c r="M15" s="21"/>
-    </row>
-    <row r="16" spans="1:13" x14ac:dyDescent="0.3">
-      <c r="C16" s="22"/>
-      <c r="D16" s="23"/>
+      <c r="H15" s="23"/>
+      <c r="I15" s="23"/>
+      <c r="J15" s="23"/>
+      <c r="K15" s="23"/>
+      <c r="L15" s="23"/>
+      <c r="M15" s="24"/>
+    </row>
+    <row r="16" spans="1:13" x14ac:dyDescent="0.25">
+      <c r="C16" s="25"/>
+      <c r="D16" s="26"/>
       <c r="F16" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G16" s="19" t="s">
+      <c r="G16" s="22" t="s">
         <v>41</v>
       </c>
-      <c r="H16" s="20"/>
-      <c r="I16" s="20"/>
-      <c r="J16" s="20"/>
-      <c r="K16" s="20"/>
-      <c r="L16" s="20"/>
-      <c r="M16" s="21"/>
-    </row>
-    <row r="17" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="H16" s="23"/>
+      <c r="I16" s="23"/>
+      <c r="J16" s="23"/>
+      <c r="K16" s="23"/>
+      <c r="L16" s="23"/>
+      <c r="M16" s="24"/>
+    </row>
+    <row r="17" spans="3:13" ht="14.45" x14ac:dyDescent="0.3">
       <c r="C17"/>
       <c r="D17"/>
       <c r="E17" s="5"/>
@@ -1036,7 +1043,7 @@
         <v>34</v>
       </c>
     </row>
-    <row r="19" spans="3:13" ht="28.8" x14ac:dyDescent="0.3">
+    <row r="19" spans="3:13" ht="30" x14ac:dyDescent="0.25">
       <c r="C19" s="6" t="s">
         <v>6</v>
       </c>
@@ -1051,7 +1058,7 @@
         <v>35</v>
       </c>
     </row>
-    <row r="20" spans="3:13" x14ac:dyDescent="0.3">
+    <row r="20" spans="3:13" ht="14.45" x14ac:dyDescent="0.3">
       <c r="C20" s="5"/>
       <c r="D20" s="5"/>
       <c r="E20" s="5"/>
@@ -1061,107 +1068,107 @@
       <c r="I20" s="5"/>
       <c r="J20" s="5"/>
     </row>
-    <row r="21" spans="3:13" ht="31.2" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C21" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="D21" s="7" t="s">
+    <row r="21" spans="3:13" ht="31.15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C21" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D21" s="11" t="s">
         <v>37</v>
       </c>
-      <c r="E21" s="5"/>
-      <c r="F21" s="3" t="s">
-        <v>0</v>
-      </c>
-      <c r="G21" s="3" t="s">
+      <c r="E21" s="27"/>
+      <c r="F21" s="12" t="s">
+        <v>0</v>
+      </c>
+      <c r="G21" s="12" t="s">
         <v>20</v>
       </c>
-      <c r="H21" s="3" t="s">
+      <c r="H21" s="12" t="s">
         <v>21</v>
       </c>
-      <c r="I21" s="3" t="s">
+      <c r="I21" s="12" t="s">
         <v>22</v>
       </c>
-      <c r="J21" s="3" t="s">
+      <c r="J21" s="12" t="s">
         <v>23</v>
       </c>
-      <c r="K21" s="3" t="s">
+      <c r="K21" s="12" t="s">
         <v>24</v>
       </c>
-      <c r="L21" s="3" t="s">
+      <c r="L21" s="12" t="s">
         <v>25</v>
       </c>
-      <c r="M21" s="3" t="s">
+      <c r="M21" s="12" t="s">
         <v>26</v>
       </c>
     </row>
-    <row r="22" spans="3:13" ht="36.6" customHeight="1" x14ac:dyDescent="0.3">
-      <c r="C22" s="16" t="s">
+    <row r="22" spans="3:13" ht="36.6" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C22" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="D22" s="17" t="s">
+      <c r="D22" s="29" t="s">
         <v>38</v>
       </c>
-      <c r="E22"/>
-      <c r="F22" s="3" t="s">
+      <c r="E22" s="30"/>
+      <c r="F22" s="12" t="s">
         <v>37</v>
       </c>
-      <c r="G22" s="3">
+      <c r="G22" s="12">
         <v>1</v>
       </c>
-      <c r="H22" s="3">
-        <v>0</v>
-      </c>
-      <c r="I22" s="3" t="s">
+      <c r="H22" s="12">
+        <v>0</v>
+      </c>
+      <c r="I22" s="12" t="s">
         <v>27</v>
       </c>
-      <c r="J22" s="3" t="s">
+      <c r="J22" s="12" t="s">
         <v>28</v>
       </c>
-      <c r="K22" s="3" t="s">
+      <c r="K22" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="L22" s="3" t="s">
+      <c r="L22" s="12" t="s">
         <v>30</v>
       </c>
-      <c r="M22" s="3">
+      <c r="M22" s="12">
         <v>15</v>
       </c>
     </row>
-    <row r="23" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C23" s="16"/>
-      <c r="D23" s="17"/>
-      <c r="E23" s="5"/>
-      <c r="F23" s="3" t="s">
+    <row r="23" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C23" s="28"/>
+      <c r="D23" s="29"/>
+      <c r="E23" s="27"/>
+      <c r="F23" s="12" t="s">
         <v>29</v>
       </c>
-      <c r="G23" s="17" t="s">
+      <c r="G23" s="29" t="s">
         <v>39</v>
       </c>
-      <c r="H23" s="17"/>
-      <c r="I23" s="17"/>
-      <c r="J23" s="17"/>
-      <c r="K23" s="17"/>
-      <c r="L23" s="17"/>
-      <c r="M23" s="17"/>
-    </row>
-    <row r="24" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C24" s="16"/>
-      <c r="D24" s="17"/>
-      <c r="E24" s="5"/>
-      <c r="F24" s="3" t="s">
+      <c r="H23" s="29"/>
+      <c r="I23" s="29"/>
+      <c r="J23" s="29"/>
+      <c r="K23" s="29"/>
+      <c r="L23" s="29"/>
+      <c r="M23" s="29"/>
+    </row>
+    <row r="24" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C24" s="28"/>
+      <c r="D24" s="29"/>
+      <c r="E24" s="27"/>
+      <c r="F24" s="12" t="s">
         <v>4</v>
       </c>
-      <c r="G24" s="17" t="s">
+      <c r="G24" s="29" t="s">
         <v>40</v>
       </c>
-      <c r="H24" s="17"/>
-      <c r="I24" s="17"/>
-      <c r="J24" s="17"/>
-      <c r="K24" s="17"/>
-      <c r="L24" s="17"/>
-      <c r="M24" s="17"/>
-    </row>
-    <row r="25" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="H24" s="29"/>
+      <c r="I24" s="29"/>
+      <c r="J24" s="29"/>
+      <c r="K24" s="29"/>
+      <c r="L24" s="29"/>
+      <c r="M24" s="29"/>
+    </row>
+    <row r="25" spans="3:13" ht="14.45" x14ac:dyDescent="0.3">
       <c r="C25" s="5"/>
       <c r="D25" s="5"/>
       <c r="E25" s="5"/>
@@ -1171,11 +1178,11 @@
       <c r="I25" s="5"/>
       <c r="J25" s="5"/>
     </row>
-    <row r="26" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C26" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="D26" s="7" t="s">
+    <row r="26" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C26" s="11" t="s">
+        <v>0</v>
+      </c>
+      <c r="D26" s="11" t="s">
         <v>43</v>
       </c>
       <c r="E26" s="5"/>
@@ -1185,12 +1192,12 @@
       <c r="I26" s="5"/>
       <c r="J26" s="5"/>
     </row>
-    <row r="27" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C27" s="16" t="s">
+    <row r="27" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C27" s="28" t="s">
         <v>6</v>
       </c>
-      <c r="D27" s="17" t="s">
-        <v>44</v>
+      <c r="D27" s="29" t="s">
+        <v>61</v>
       </c>
       <c r="E27" s="5"/>
       <c r="F27" s="5"/>
@@ -1199,9 +1206,9 @@
       <c r="I27" s="5"/>
       <c r="J27" s="5"/>
     </row>
-    <row r="28" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C28" s="16"/>
-      <c r="D28" s="17"/>
+    <row r="28" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C28" s="28"/>
+      <c r="D28" s="29"/>
       <c r="E28" s="5"/>
       <c r="F28" s="5"/>
       <c r="G28" s="5"/>
@@ -1209,9 +1216,9 @@
       <c r="I28" s="5"/>
       <c r="J28" s="5"/>
     </row>
-    <row r="29" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C29" s="16"/>
-      <c r="D29" s="17"/>
+    <row r="29" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C29" s="28"/>
+      <c r="D29" s="29"/>
       <c r="E29" s="5"/>
       <c r="F29" s="5"/>
       <c r="G29" s="5"/>
@@ -1219,7 +1226,7 @@
       <c r="I29" s="5"/>
       <c r="J29" s="5"/>
     </row>
-    <row r="30" spans="3:13" x14ac:dyDescent="0.3">
+    <row r="30" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C30" s="5"/>
       <c r="D30" s="5"/>
       <c r="E30" s="5"/>
@@ -1229,43 +1236,49 @@
       <c r="I30" s="5"/>
       <c r="J30" s="5"/>
     </row>
-    <row r="31" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C31" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="D31" s="7" t="s">
+    <row r="31" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C31" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D31" s="16" t="s">
         <v>45</v>
       </c>
       <c r="E31" s="5"/>
-      <c r="F31" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="G31" s="7" t="s">
-        <v>47</v>
+      <c r="F31" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="G31" s="16" t="s">
+        <v>46</v>
       </c>
       <c r="H31" s="5"/>
       <c r="I31" s="5"/>
       <c r="J31" s="5"/>
-    </row>
-    <row r="32" spans="3:13" ht="43.2" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K31" s="18"/>
+      <c r="L31" s="18"/>
+      <c r="M31" s="18"/>
+    </row>
+    <row r="32" spans="3:13" ht="43.15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C32" s="16" t="s">
         <v>6</v>
       </c>
       <c r="D32" s="17" t="s">
-        <v>61</v>
+        <v>47</v>
       </c>
       <c r="E32" s="5"/>
       <c r="F32" s="16" t="s">
         <v>6</v>
       </c>
       <c r="G32" s="17" t="s">
-        <v>48</v>
+        <v>62</v>
       </c>
       <c r="H32" s="5"/>
       <c r="I32" s="5"/>
       <c r="J32" s="5"/>
-    </row>
-    <row r="33" spans="3:13" ht="15" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K32" s="18"/>
+      <c r="L32" s="18"/>
+      <c r="M32" s="18"/>
+    </row>
+    <row r="33" spans="3:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C33" s="16"/>
       <c r="D33" s="17"/>
       <c r="E33" s="5"/>
@@ -1274,8 +1287,11 @@
       <c r="H33" s="5"/>
       <c r="I33" s="5"/>
       <c r="J33" s="5"/>
-    </row>
-    <row r="34" spans="3:13" ht="32.4" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="K33" s="18"/>
+      <c r="L33" s="18"/>
+      <c r="M33" s="18"/>
+    </row>
+    <row r="34" spans="3:13" ht="32.450000000000003" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C34" s="16"/>
       <c r="D34" s="17"/>
       <c r="E34" s="5"/>
@@ -1284,8 +1300,11 @@
       <c r="H34" s="5"/>
       <c r="I34" s="5"/>
       <c r="J34" s="5"/>
-    </row>
-    <row r="35" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="K34" s="18"/>
+      <c r="L34" s="18"/>
+      <c r="M34" s="18"/>
+    </row>
+    <row r="35" spans="3:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C35" s="5"/>
       <c r="D35" s="5"/>
       <c r="E35" s="5"/>
@@ -1294,64 +1313,111 @@
       <c r="H35" s="5"/>
       <c r="I35" s="5"/>
       <c r="J35" s="5"/>
-    </row>
-    <row r="36" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C36" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="D36" s="7" t="s">
-        <v>49</v>
+      <c r="K35" s="18"/>
+      <c r="L35" s="18"/>
+      <c r="M35" s="18"/>
+    </row>
+    <row r="36" spans="3:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C36" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D36" s="16" t="s">
+        <v>48</v>
       </c>
       <c r="E36" s="5"/>
-      <c r="F36" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="G36" s="7" t="s">
-        <v>50</v>
-      </c>
-      <c r="H36" s="5"/>
-      <c r="I36" s="5"/>
-      <c r="J36" s="5"/>
-    </row>
-    <row r="37" spans="3:13" ht="28.8" customHeight="1" x14ac:dyDescent="0.3">
+      <c r="F36" s="17" t="s">
+        <v>0</v>
+      </c>
+      <c r="G36" s="17" t="s">
+        <v>20</v>
+      </c>
+      <c r="H36" s="17" t="s">
+        <v>21</v>
+      </c>
+      <c r="I36" s="17" t="s">
+        <v>22</v>
+      </c>
+      <c r="J36" s="17" t="s">
+        <v>23</v>
+      </c>
+      <c r="K36" s="17" t="s">
+        <v>24</v>
+      </c>
+      <c r="L36" s="17" t="s">
+        <v>25</v>
+      </c>
+      <c r="M36" s="17" t="s">
+        <v>26</v>
+      </c>
+    </row>
+    <row r="37" spans="3:13" ht="28.9" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C37" s="16" t="s">
         <v>6</v>
       </c>
       <c r="D37" s="17" t="s">
+        <v>52</v>
+      </c>
+      <c r="E37" s="5"/>
+      <c r="F37" s="17" t="s">
+        <v>53</v>
+      </c>
+      <c r="G37" s="17" t="s">
+        <v>49</v>
+      </c>
+      <c r="H37" s="17" t="s">
+        <v>50</v>
+      </c>
+      <c r="I37" s="17" t="s">
+        <v>58</v>
+      </c>
+      <c r="J37" s="17" t="s">
+        <v>28</v>
+      </c>
+      <c r="K37" s="17" t="s">
         <v>51</v>
       </c>
-      <c r="E37" s="5"/>
-      <c r="F37" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="G37" s="17" t="s">
-        <v>52</v>
-      </c>
-      <c r="H37" s="5"/>
-      <c r="I37" s="5"/>
-      <c r="J37" s="5"/>
-    </row>
-    <row r="38" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="L37" s="17" t="s">
+        <v>51</v>
+      </c>
+      <c r="M37" s="17">
+        <v>20</v>
+      </c>
+    </row>
+    <row r="38" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C38" s="16"/>
       <c r="D38" s="17"/>
       <c r="E38" s="5"/>
-      <c r="F38" s="16"/>
-      <c r="G38" s="17"/>
-      <c r="H38" s="5"/>
-      <c r="I38" s="5"/>
-      <c r="J38" s="5"/>
-    </row>
-    <row r="39" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F38" s="17" t="s">
+        <v>29</v>
+      </c>
+      <c r="G38" s="17" t="s">
+        <v>54</v>
+      </c>
+      <c r="H38" s="17"/>
+      <c r="I38" s="17"/>
+      <c r="J38" s="17"/>
+      <c r="K38" s="17"/>
+      <c r="L38" s="17"/>
+      <c r="M38" s="17"/>
+    </row>
+    <row r="39" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C39" s="16"/>
       <c r="D39" s="17"/>
       <c r="E39" s="5"/>
-      <c r="F39" s="16"/>
-      <c r="G39" s="17"/>
-      <c r="H39" s="5"/>
-      <c r="I39" s="5"/>
-      <c r="J39" s="5"/>
-    </row>
-    <row r="40" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F39" s="17" t="s">
+        <v>4</v>
+      </c>
+      <c r="G39" s="17" t="s">
+        <v>55</v>
+      </c>
+      <c r="H39" s="17"/>
+      <c r="I39" s="17"/>
+      <c r="J39" s="17"/>
+      <c r="K39" s="17"/>
+      <c r="L39" s="17"/>
+      <c r="M39" s="17"/>
+    </row>
+    <row r="40" spans="3:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C40" s="5"/>
       <c r="D40" s="5"/>
       <c r="E40" s="5"/>
@@ -1360,41 +1426,28 @@
       <c r="H40" s="5"/>
       <c r="I40" s="5"/>
       <c r="J40" s="5"/>
-    </row>
-    <row r="41" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C41" s="7" t="s">
-        <v>0</v>
-      </c>
-      <c r="D41" s="7" t="s">
-        <v>53</v>
+      <c r="K40" s="18"/>
+      <c r="L40" s="18"/>
+      <c r="M40" s="18"/>
+    </row>
+    <row r="41" spans="3:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C41" s="16" t="s">
+        <v>0</v>
+      </c>
+      <c r="D41" s="16" t="s">
+        <v>56</v>
       </c>
       <c r="E41" s="5"/>
-      <c r="F41" s="13" t="s">
-        <v>0</v>
-      </c>
-      <c r="G41" s="13" t="s">
-        <v>20</v>
-      </c>
-      <c r="H41" s="13" t="s">
-        <v>21</v>
-      </c>
-      <c r="I41" s="13" t="s">
-        <v>22</v>
-      </c>
-      <c r="J41" s="13" t="s">
-        <v>23</v>
-      </c>
-      <c r="K41" s="13" t="s">
-        <v>24</v>
-      </c>
-      <c r="L41" s="13" t="s">
-        <v>25</v>
-      </c>
-      <c r="M41" s="13" t="s">
-        <v>26</v>
-      </c>
-    </row>
-    <row r="42" spans="3:13" ht="28.8" x14ac:dyDescent="0.3">
+      <c r="F41" s="5"/>
+      <c r="G41" s="5"/>
+      <c r="H41" s="5"/>
+      <c r="I41" s="5"/>
+      <c r="J41" s="5"/>
+      <c r="K41" s="18"/>
+      <c r="L41" s="18"/>
+      <c r="M41" s="18"/>
+    </row>
+    <row r="42" spans="3:13" ht="30" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C42" s="16" t="s">
         <v>6</v>
       </c>
@@ -1402,66 +1455,42 @@
         <v>57</v>
       </c>
       <c r="E42" s="5"/>
-      <c r="F42" s="13" t="s">
-        <v>58</v>
-      </c>
-      <c r="G42" s="13" t="s">
-        <v>54</v>
-      </c>
-      <c r="H42" s="13" t="s">
-        <v>55</v>
-      </c>
-      <c r="I42" s="13" t="s">
-        <v>64</v>
-      </c>
-      <c r="J42" s="13" t="s">
-        <v>28</v>
-      </c>
-      <c r="K42" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="L42" s="13" t="s">
-        <v>56</v>
-      </c>
-      <c r="M42" s="13">
-        <v>20</v>
-      </c>
-    </row>
-    <row r="43" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F42" s="5"/>
+      <c r="G42" s="5"/>
+      <c r="H42" s="5"/>
+      <c r="I42" s="5"/>
+      <c r="J42" s="5"/>
+      <c r="K42" s="18"/>
+      <c r="L42" s="18"/>
+      <c r="M42" s="18"/>
+    </row>
+    <row r="43" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C43" s="16"/>
       <c r="D43" s="17"/>
       <c r="E43" s="5"/>
-      <c r="F43" s="13" t="s">
-        <v>29</v>
-      </c>
-      <c r="G43" s="17" t="s">
-        <v>59</v>
-      </c>
-      <c r="H43" s="17"/>
-      <c r="I43" s="17"/>
-      <c r="J43" s="17"/>
-      <c r="K43" s="17"/>
-      <c r="L43" s="17"/>
-      <c r="M43" s="17"/>
-    </row>
-    <row r="44" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F43" s="5"/>
+      <c r="G43" s="5"/>
+      <c r="H43" s="5"/>
+      <c r="I43" s="5"/>
+      <c r="J43" s="5"/>
+      <c r="K43" s="18"/>
+      <c r="L43" s="18"/>
+      <c r="M43" s="18"/>
+    </row>
+    <row r="44" spans="3:13" x14ac:dyDescent="0.25">
       <c r="C44" s="16"/>
       <c r="D44" s="17"/>
       <c r="E44" s="5"/>
-      <c r="F44" s="13" t="s">
-        <v>4</v>
-      </c>
-      <c r="G44" s="17" t="s">
-        <v>60</v>
-      </c>
-      <c r="H44" s="17"/>
-      <c r="I44" s="17"/>
-      <c r="J44" s="17"/>
-      <c r="K44" s="17"/>
-      <c r="L44" s="17"/>
-      <c r="M44" s="17"/>
-    </row>
-    <row r="45" spans="3:13" x14ac:dyDescent="0.3">
+      <c r="F44" s="5"/>
+      <c r="G44" s="5"/>
+      <c r="H44" s="5"/>
+      <c r="I44" s="5"/>
+      <c r="J44" s="5"/>
+      <c r="K44" s="18"/>
+      <c r="L44" s="18"/>
+      <c r="M44" s="18"/>
+    </row>
+    <row r="45" spans="3:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C45" s="5"/>
       <c r="D45" s="5"/>
       <c r="E45" s="5"/>
@@ -1471,12 +1500,12 @@
       <c r="I45" s="5"/>
       <c r="J45" s="5"/>
     </row>
-    <row r="46" spans="3:13" x14ac:dyDescent="0.3">
+    <row r="46" spans="3:13" ht="14.45" customHeight="1" x14ac:dyDescent="0.25">
       <c r="C46" s="14" t="s">
         <v>0</v>
       </c>
       <c r="D46" s="14" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
       <c r="E46" s="5"/>
       <c r="F46" s="5"/>
@@ -1485,12 +1514,12 @@
       <c r="I46" s="5"/>
       <c r="J46" s="5"/>
     </row>
-    <row r="47" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C47" s="16" t="s">
+    <row r="47" spans="3:13" ht="15" customHeight="1" x14ac:dyDescent="0.25">
+      <c r="C47" s="19" t="s">
         <v>6</v>
       </c>
-      <c r="D47" s="17" t="s">
-        <v>63</v>
+      <c r="D47" s="20" t="s">
+        <v>60</v>
       </c>
       <c r="E47" s="5"/>
       <c r="F47" s="5"/>
@@ -1499,9 +1528,9 @@
       <c r="I47" s="5"/>
       <c r="J47" s="5"/>
     </row>
-    <row r="48" spans="3:13" x14ac:dyDescent="0.3">
-      <c r="C48" s="16"/>
-      <c r="D48" s="17"/>
+    <row r="48" spans="3:13" x14ac:dyDescent="0.25">
+      <c r="C48" s="19"/>
+      <c r="D48" s="20"/>
       <c r="E48" s="5"/>
       <c r="F48" s="5"/>
       <c r="G48" s="5"/>
@@ -1509,9 +1538,9 @@
       <c r="I48" s="5"/>
       <c r="J48" s="5"/>
     </row>
-    <row r="49" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C49" s="16"/>
-      <c r="D49" s="17"/>
+    <row r="49" spans="3:10" x14ac:dyDescent="0.25">
+      <c r="C49" s="19"/>
+      <c r="D49" s="20"/>
       <c r="E49" s="5"/>
       <c r="F49" s="5"/>
       <c r="G49" s="5"/>
@@ -1519,65 +1548,7 @@
       <c r="I49" s="5"/>
       <c r="J49" s="5"/>
     </row>
-    <row r="50" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C50" s="5"/>
-      <c r="D50" s="5"/>
-      <c r="E50" s="5"/>
-      <c r="F50" s="5"/>
-      <c r="G50" s="5"/>
-      <c r="H50" s="5"/>
-      <c r="I50" s="5"/>
-      <c r="J50" s="5"/>
-    </row>
-    <row r="51" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C51" s="14" t="s">
-        <v>0</v>
-      </c>
-      <c r="D51" s="14" t="s">
-        <v>65</v>
-      </c>
-      <c r="E51" s="5"/>
-      <c r="F51" s="5"/>
-      <c r="G51" s="5"/>
-      <c r="H51" s="5"/>
-      <c r="I51" s="5"/>
-      <c r="J51" s="5"/>
-    </row>
-    <row r="52" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C52" s="16" t="s">
-        <v>6</v>
-      </c>
-      <c r="D52" s="17" t="s">
-        <v>66</v>
-      </c>
-      <c r="E52" s="5"/>
-      <c r="F52" s="5"/>
-      <c r="G52" s="5"/>
-      <c r="H52" s="5"/>
-      <c r="I52" s="5"/>
-      <c r="J52" s="5"/>
-    </row>
-    <row r="53" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C53" s="16"/>
-      <c r="D53" s="17"/>
-      <c r="E53" s="5"/>
-      <c r="F53" s="5"/>
-      <c r="G53" s="5"/>
-      <c r="H53" s="5"/>
-      <c r="I53" s="5"/>
-      <c r="J53" s="5"/>
-    </row>
-    <row r="54" spans="3:10" x14ac:dyDescent="0.3">
-      <c r="C54" s="16"/>
-      <c r="D54" s="17"/>
-      <c r="E54" s="5"/>
-      <c r="F54" s="5"/>
-      <c r="G54" s="5"/>
-      <c r="H54" s="5"/>
-      <c r="I54" s="5"/>
-      <c r="J54" s="5"/>
-    </row>
-    <row r="55" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="55" spans="3:10" x14ac:dyDescent="0.25">
       <c r="C55" s="5"/>
       <c r="D55" s="5"/>
       <c r="E55" s="5"/>
@@ -1587,7 +1558,7 @@
       <c r="I55" s="5"/>
       <c r="J55" s="5"/>
     </row>
-    <row r="56" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="56" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
       <c r="C56" s="5"/>
       <c r="D56" s="5"/>
       <c r="E56" s="5"/>
@@ -1597,7 +1568,7 @@
       <c r="I56" s="5"/>
       <c r="J56" s="5"/>
     </row>
-    <row r="57" spans="3:10" x14ac:dyDescent="0.3">
+    <row r="57" spans="3:10" ht="14.45" x14ac:dyDescent="0.3">
       <c r="C57" s="5"/>
       <c r="D57" s="5"/>
       <c r="E57" s="5"/>
@@ -1607,7 +1578,7 @@
       <c r="I57" s="5"/>
       <c r="J57" s="5"/>
     </row>
-    <row r="58" spans="3:10" ht="55.2" customHeight="1" x14ac:dyDescent="0.3">
+    <row r="58" spans="3:10" ht="55.15" customHeight="1" x14ac:dyDescent="0.3">
       <c r="C58" s="5"/>
       <c r="D58" s="5"/>
       <c r="E58" s="5"/>
@@ -1618,35 +1589,21 @@
       <c r="J58" s="5"/>
     </row>
   </sheetData>
-  <mergeCells count="28">
-    <mergeCell ref="C47:C49"/>
-    <mergeCell ref="D47:D49"/>
-    <mergeCell ref="C52:C54"/>
-    <mergeCell ref="D52:D54"/>
-    <mergeCell ref="C27:C29"/>
-    <mergeCell ref="D27:D29"/>
-    <mergeCell ref="C32:C34"/>
-    <mergeCell ref="D32:D34"/>
-    <mergeCell ref="F1:L1"/>
-    <mergeCell ref="F32:F34"/>
-    <mergeCell ref="G32:G34"/>
-    <mergeCell ref="G23:M23"/>
-    <mergeCell ref="G24:M24"/>
+  <mergeCells count="14">
+    <mergeCell ref="D22:D24"/>
+    <mergeCell ref="C22:C24"/>
     <mergeCell ref="A1:E1"/>
     <mergeCell ref="G15:M15"/>
     <mergeCell ref="G16:M16"/>
     <mergeCell ref="C14:C16"/>
     <mergeCell ref="D14:D16"/>
-    <mergeCell ref="D22:D24"/>
-    <mergeCell ref="C22:C24"/>
-    <mergeCell ref="C37:C39"/>
-    <mergeCell ref="D37:D39"/>
-    <mergeCell ref="F37:F39"/>
-    <mergeCell ref="G37:G39"/>
-    <mergeCell ref="C42:C44"/>
-    <mergeCell ref="D42:D44"/>
-    <mergeCell ref="G43:M43"/>
-    <mergeCell ref="G44:M44"/>
+    <mergeCell ref="F1:L1"/>
+    <mergeCell ref="G23:M23"/>
+    <mergeCell ref="G24:M24"/>
+    <mergeCell ref="C47:C49"/>
+    <mergeCell ref="D47:D49"/>
+    <mergeCell ref="C27:C29"/>
+    <mergeCell ref="D27:D29"/>
   </mergeCells>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
   <pageSetup paperSize="9" orientation="portrait" r:id="rId1"/>
@@ -1656,9 +1613,9 @@
 <file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
-    <col min="3" max="3" width="12.5546875" customWidth="1"/>
+    <col min="3" max="3" width="12.5703125" customWidth="1"/>
   </cols>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
@@ -1668,7 +1625,7 @@
 <file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" mc:Ignorable="x14ac">
   <dimension ref="A1"/>
-  <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
+  <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <sheetData/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>